<commit_message>
Added paragraph 3 divided in private and public
</commit_message>
<xml_diff>
--- a/Table_S2.xlsx
+++ b/Table_S2.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">Scheme</t>
   </si>
@@ -48,6 +48,12 @@
   </si>
   <si>
     <t xml:space="preserve">Game reserve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Article3, Private</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Article3, Public</t>
   </si>
   <si>
     <t xml:space="preserve">Dune protection scheme</t>
@@ -506,28 +512,28 @@
         <v>12</v>
       </c>
       <c r="B5" t="n">
-        <v>159.4856</v>
+        <v>3138.7962</v>
       </c>
       <c r="C5" t="n">
-        <v>0.369651549873695</v>
+        <v>7.27501968872215</v>
       </c>
       <c r="D5" t="n">
-        <v>3.9058</v>
+        <v>49.5792</v>
       </c>
       <c r="E5" t="n">
-        <v>2.44899853027483</v>
+        <v>1.57956097946085</v>
       </c>
       <c r="F5" t="n">
-        <v>24.9032</v>
+        <v>1375.5933</v>
       </c>
       <c r="G5" t="n">
-        <v>15.6147012645656</v>
+        <v>43.8255054597046</v>
       </c>
       <c r="H5" t="n">
-        <v>4.1009</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>2.57132932377594</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -535,22 +541,22 @@
         <v>13</v>
       </c>
       <c r="B6" t="n">
-        <v>21.3049</v>
+        <v>1079.9861</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0493799396616628</v>
+        <v>2.50316351888226</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9924</v>
+        <v>20.3492</v>
       </c>
       <c r="E6" t="n">
-        <v>4.65808335171721</v>
+        <v>1.88420943565848</v>
       </c>
       <c r="F6" t="n">
-        <v>2.0805</v>
+        <v>341.5356</v>
       </c>
       <c r="G6" t="n">
-        <v>9.76535914273243</v>
+        <v>31.6240736802075</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -564,27 +570,85 @@
         <v>14</v>
       </c>
       <c r="B7" t="n">
+        <v>159.4856</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.369651549873695</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3.9058</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2.44899853027483</v>
+      </c>
+      <c r="F7" t="n">
+        <v>24.9032</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15.6147012645656</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4.1009</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.57132932377594</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="n">
+        <v>21.3049</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0493799396616628</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.9924</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.65808335171721</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.0805</v>
+      </c>
+      <c r="G8" t="n">
+        <v>9.76535914273243</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="n">
         <v>247.0934</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C9" t="n">
         <v>0.572706615980132</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D9" t="n">
         <v>4.8253</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E9" t="n">
         <v>1.95282431663492</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F9" t="n">
         <v>78.2871</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G9" t="n">
         <v>31.6832015747891</v>
       </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added untouched forest to the table
</commit_message>
<xml_diff>
--- a/Table_S2.xlsx
+++ b/Table_S2.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Scheme</t>
   </si>
@@ -54,6 +54,12 @@
   </si>
   <si>
     <t xml:space="preserve">Article3, Public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unmanaged_Forest_Sate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unmanaged_Forest_Private</t>
   </si>
   <si>
     <t xml:space="preserve">Dune protection scheme</t>
@@ -570,28 +576,28 @@
         <v>14</v>
       </c>
       <c r="B7" t="n">
-        <v>159.4856</v>
+        <v>484.7643</v>
       </c>
       <c r="C7" t="n">
-        <v>0.369651549873695</v>
+        <v>1.12357400805112</v>
       </c>
       <c r="D7" t="n">
-        <v>3.9058</v>
+        <v>16.6381</v>
       </c>
       <c r="E7" t="n">
-        <v>2.44899853027483</v>
+        <v>3.43220406288169</v>
       </c>
       <c r="F7" t="n">
-        <v>24.9032</v>
+        <v>31.7915</v>
       </c>
       <c r="G7" t="n">
-        <v>15.6147012645656</v>
+        <v>6.55813557227708</v>
       </c>
       <c r="H7" t="n">
-        <v>4.1009</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2.57132932377594</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -599,22 +605,22 @@
         <v>15</v>
       </c>
       <c r="B8" t="n">
-        <v>21.3049</v>
+        <v>26.784</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0493799396616628</v>
+        <v>0.0620792542512745</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9924</v>
+        <v>0.6454</v>
       </c>
       <c r="E8" t="n">
-        <v>4.65808335171721</v>
+        <v>2.40964755077658</v>
       </c>
       <c r="F8" t="n">
-        <v>2.0805</v>
+        <v>1.0794</v>
       </c>
       <c r="G8" t="n">
-        <v>9.76535914273243</v>
+        <v>4.03001792114695</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -628,27 +634,85 @@
         <v>16</v>
       </c>
       <c r="B9" t="n">
+        <v>159.4856</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.369651549873695</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3.9058</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.44899853027483</v>
+      </c>
+      <c r="F9" t="n">
+        <v>24.9032</v>
+      </c>
+      <c r="G9" t="n">
+        <v>15.6147012645656</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4.1009</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.57132932377594</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="n">
+        <v>21.3049</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0493799396616628</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9924</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.65808335171721</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.0805</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9.76535914273243</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="n">
         <v>247.0934</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C11" t="n">
         <v>0.572706615980132</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D11" t="n">
         <v>4.8253</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E11" t="n">
         <v>1.95282431663492</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F11" t="n">
         <v>78.2871</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G11" t="n">
         <v>31.6832015747891</v>
       </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Took out PGR, from agriculture
</commit_message>
<xml_diff>
--- a/Table_S2.xlsx
+++ b/Table_S2.xlsx
@@ -443,10 +443,10 @@
         <v>3.77638963797406</v>
       </c>
       <c r="F2" t="n">
-        <v>1561.0322</v>
+        <v>698.7227</v>
       </c>
       <c r="G2" t="n">
-        <v>40.2471043888575</v>
+        <v>18.0147247736237</v>
       </c>
       <c r="H2" t="n">
         <v>447.4382</v>
@@ -472,10 +472,10 @@
         <v>3.67779808399777</v>
       </c>
       <c r="F3" t="n">
-        <v>433.4139</v>
+        <v>246.0695</v>
       </c>
       <c r="G3" t="n">
-        <v>39.6977807966908</v>
+        <v>22.5383013137126</v>
       </c>
       <c r="H3" t="n">
         <v>108.7341</v>
@@ -530,10 +530,10 @@
         <v>1.57956097946085</v>
       </c>
       <c r="F5" t="n">
-        <v>1375.5933</v>
+        <v>981.6512</v>
       </c>
       <c r="G5" t="n">
-        <v>43.8255054597046</v>
+        <v>31.2747670587852</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -559,10 +559,10 @@
         <v>1.88420943565848</v>
       </c>
       <c r="F6" t="n">
-        <v>341.5356</v>
+        <v>276.1203</v>
       </c>
       <c r="G6" t="n">
-        <v>31.6240736802075</v>
+        <v>25.5670235015062</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         <v>3.43220406288169</v>
       </c>
       <c r="F7" t="n">
-        <v>31.7915</v>
+        <v>23.7362</v>
       </c>
       <c r="G7" t="n">
-        <v>6.55813557227708</v>
+        <v>4.89644142524522</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -617,10 +617,10 @@
         <v>2.40964755077658</v>
       </c>
       <c r="F8" t="n">
-        <v>1.0794</v>
+        <v>0.3731</v>
       </c>
       <c r="G8" t="n">
-        <v>4.03001792114695</v>
+        <v>1.39299581839904</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -646,10 +646,10 @@
         <v>2.44899853027483</v>
       </c>
       <c r="F9" t="n">
-        <v>24.9032</v>
+        <v>20.7219</v>
       </c>
       <c r="G9" t="n">
-        <v>15.6147012645656</v>
+        <v>12.9929598659691</v>
       </c>
       <c r="H9" t="n">
         <v>4.1009</v>
@@ -675,10 +675,10 @@
         <v>4.65808335171721</v>
       </c>
       <c r="F10" t="n">
-        <v>2.0805</v>
+        <v>0.9185</v>
       </c>
       <c r="G10" t="n">
-        <v>9.76535914273243</v>
+        <v>4.31121479096358</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -704,10 +704,10 @@
         <v>1.95282431663492</v>
       </c>
       <c r="F11" t="n">
-        <v>78.2871</v>
+        <v>32.7739</v>
       </c>
       <c r="G11" t="n">
-        <v>31.6832015747891</v>
+        <v>13.2637698942991</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>

</xml_diff>